<commit_message>
No variance bullet under $1K, and fix the Roosevelt August draft
Emma flagged that the Roosevelt Commons August commentary was full of sub-$1K
bullets. Six of them, "-$0.1K Pest Control Maintenance, Sweeping" being the
worst. Small accounts are now grouped until each line clears $1,000 with every
account named, which is how Athena's own summaries read.

Grouped, not dropped. Every group re-checked against its headline: income
month, operating expenses month and year, owner expenses month and year all
tie exactly.

The rule was only written loosely before, HOW-IT-WORKS.md said items "under a
few hundred dollars can be left off". Now stated as a $1K floor in both
HOW-IT-WORKS.md and WORKFLOW.md, with Athena's own grouped bullets as the
examples, so it holds next month.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu4BYRooeTwe4PF531ukub
</commit_message>
<xml_diff>
--- a/tasks/monthly-reports/outbox/2026-09-08-RSC-august-2026-executive-summary.xlsx
+++ b/tasks/monthly-reports/outbox/2026-09-08-RSC-august-2026-executive-summary.xlsx
@@ -2782,8 +2782,7 @@
 -$1.1K Desert Financial Credit Union, Someburros, Pita Kitchen, Port of Subs
 Offset by:
 -($12.7K) McDonald's, short payment on base rent and NNN
--($9.1K) The Buffalo Spot, no payment
--($0.6K) TA Nail Bar, Panda Express</t>
+-($9.7K) The Buffalo Spot no payment, TA Nail Bar, Panda Express</t>
         </is>
       </c>
       <c r="B21" s="121"/>
@@ -2843,15 +2842,12 @@
         <is>
           <t xml:space="preserve">MTD Operating Expenses are under budget by $2,633.68 or 14.19% due to:
 -$2K Water/Building
+-$2K Trash Removal, Electric/Building, Electric/Common Area, Pest Control Maintenance, Sweeping
 -$1.5K Water/Common Area
 -$1.3K Sidewalk Maintenance
--$1.1K Trash Removal
--$0.8K Electric/Building, Electric/Common Area
--$0.1K Pest Control Maintenance, Sweeping
 Offset by:
--($1.8K) Landscape - Tree Trimmings
--($1.4K) On Site Management Fees
--($0.9K) Janitorial, Building Lighting Maintenance &amp; Repairs</t>
+-($2.3K) On Site Management Fees, Janitorial, Building Lighting Maintenance &amp; Repairs
+-($1.8K) Landscape - Tree Trimmings</t>
         </is>
       </c>
       <c r="B24" s="122"/>
@@ -2883,13 +2879,11 @@
 -$2.4K Water/Common Area
 -$2.2K Sidewalk Maintenance
 -$2.1K Water/Building
--$0.9K Electric/Building
--$1.8K Electric/Common Area, Insurance - Umbrella, Trash Removal, Monitor Fire Sprinklers, Landscape - Sprinkler Repairs, Pest Control Maintenance
+-$2.7K Electric/Building, Electric/Common Area, Insurance - Umbrella, Trash Removal, Monitor Fire Sprinklers, Landscape - Sprinkler Repairs, Pest Control Maintenance
 Offset by:
 -($15.6K) Insurance - Property
--($1.8K) Landscape - Tree Trimmings
--($1.6K) Landscape - Maintenance
--($0.5K) On Site Management Fees, Janitorial, Building Lighting Maintenance &amp; Repairs</t>
+-($2.1K) Landscape - Maintenance, On Site Management Fees, Janitorial, Building Lighting Maintenance &amp; Repairs
+-($1.8K) Landscape - Tree Trimmings</t>
         </is>
       </c>
       <c r="B25" s="123"/>

</xml_diff>